<commit_message>
phase2: launch 30-day sprint plan, audit template, and restructure daily tasks
- Add phase2_plan.md: 30-day actionable plan (5 to 50+ products)
- Add phase2_audit.md: project health check template
- Remove day_03 ~ day_56 (Phase 1 completed, consolidated into Phase 2)
- Add new output subdirs: detail_pages/, seo_titles/, rfq_reply/, whatsapp_scripts/
- Add input PDF, CSV database, and processed products metadata
</commit_message>
<xml_diff>
--- a/04-database/templates/product_database_template.xlsx
+++ b/04-database/templates/product_database_template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\AI-外贸自动化系统\01-产品数据库模板\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\code\05_AI-外贸自动化系统\04-database\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C65922C4-9A37-42C8-BE9E-DCD0C7F9A2FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E2A7D8-CDE6-4B24-97CA-EC8D911E3850}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>product_id</t>
   </si>
@@ -113,237 +113,6 @@
   </si>
   <si>
     <t>alibaba_detail_status</t>
-  </si>
-  <si>
-    <t>GF-001</t>
-  </si>
-  <si>
-    <t>园林叉</t>
-  </si>
-  <si>
-    <t>Garden Fork</t>
-  </si>
-  <si>
-    <t>Digging Tools</t>
-  </si>
-  <si>
-    <t>Forks</t>
-  </si>
-  <si>
-    <t>Carbon Steel + Ash Wood</t>
-  </si>
-  <si>
-    <t>Ash Wood</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>0.8</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>HRC 45-50</t>
-  </si>
-  <si>
-    <t>Polished + Lacquered</t>
-  </si>
-  <si>
-    <t>Color Box</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>62x32x35</t>
-  </si>
-  <si>
-    <t>17.5</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>CE, GS</t>
-  </si>
-  <si>
-    <t>garden fork, digging fork, steel fork</t>
-  </si>
-  <si>
-    <t>Garden soil turning, compost mixing, lawn aeration</t>
-  </si>
-  <si>
-    <t>Europe, Africa, South America</t>
-  </si>
-  <si>
-    <t>Extra-strong tines, ergonomic ash wood handle</t>
-  </si>
-  <si>
-    <t>Fiskars X3, Spear &amp; Jackson</t>
-  </si>
-  <si>
-    <t>pending</t>
-  </si>
-  <si>
-    <t>GS-001</t>
-  </si>
-  <si>
-    <t>园林铲</t>
-  </si>
-  <si>
-    <t>Garden Spade</t>
-  </si>
-  <si>
-    <t>Spades</t>
-  </si>
-  <si>
-    <t>Carbon Steel + Hardwood</t>
-  </si>
-  <si>
-    <t>Hardwood (FSC Certified)</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>0.6</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>HRC 42-48</t>
-  </si>
-  <si>
-    <t>Painted + Epoxy Coated</t>
-  </si>
-  <si>
-    <t>72x28x20</t>
-  </si>
-  <si>
-    <t>16.0</t>
-  </si>
-  <si>
-    <t>CE, GS, FSC</t>
-  </si>
-  <si>
-    <t>garden spade, digging spade, transplanting shovel</t>
-  </si>
-  <si>
-    <t>Transplanting, edging, trenching, soil digging</t>
-  </si>
-  <si>
-    <t>Europe, North America, Australia</t>
-  </si>
-  <si>
-    <t>FSC certified wood handle, lightweight yet strong</t>
-  </si>
-  <si>
-    <t>Burgon &amp; Ball, Bulldog</t>
-  </si>
-  <si>
-    <t>GR-001</t>
-  </si>
-  <si>
-    <t>园林耙</t>
-  </si>
-  <si>
-    <t>Garden Rake</t>
-  </si>
-  <si>
-    <t>Rakes</t>
-  </si>
-  <si>
-    <t>Carbon Steel + Wooden Handle</t>
-  </si>
-  <si>
-    <t>Wooden Handle</t>
-  </si>
-  <si>
-    <t>35</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>HRC 40-45</t>
-  </si>
-  <si>
-    <t>Polished</t>
-  </si>
-  <si>
-    <t>Blister Card</t>
-  </si>
-  <si>
-    <t>CE</t>
-  </si>
-  <si>
-    <t>garden rake, leaf rake, steel rake, lawn rake</t>
-  </si>
-  <si>
-    <t>Leaf gathering, soil leveling, debris clearing</t>
-  </si>
-  <si>
-    <t>Europe, North America, Japan</t>
-  </si>
-  <si>
-    <t>14-tine design for efficient gathering, lightweight</t>
-  </si>
-  <si>
-    <t>Ames, Corona</t>
-  </si>
-  <si>
-    <t>HT-001</t>
-  </si>
-  <si>
-    <t>园艺锄</t>
-  </si>
-  <si>
-    <t>Garden Hoe</t>
-  </si>
-  <si>
-    <t>Weeding Tools</t>
-  </si>
-  <si>
-    <t>Hoes</t>
-  </si>
-  <si>
-    <t>Hardwood</t>
-  </si>
-  <si>
-    <t>0.7</t>
-  </si>
-  <si>
-    <t>Polished + Anti-rust coating</t>
-  </si>
-  <si>
-    <t>Hang Card</t>
-  </si>
-  <si>
-    <t>72x38x10</t>
-  </si>
-  <si>
-    <t>15.0</t>
-  </si>
-  <si>
-    <t>garden hoe, weeding hoe, steel hoe</t>
-  </si>
-  <si>
-    <t>Weeding, soil breaking, row making</t>
-  </si>
-  <si>
-    <t>Africa, South America, Southeast Asia</t>
-  </si>
-  <si>
-    <t>Sharp blade for easy weeding, durable coating</t>
-  </si>
-  <si>
-    <t>True Temper, Rogue</t>
-  </si>
-  <si>
-    <t>43x43x18</t>
   </si>
 </sst>
 </file>
@@ -738,7 +507,7 @@
     <col min="16" max="31" width="18.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:31" s="2" customFormat="1" ht="30" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -834,334 +603,134 @@
       </c>
     </row>
     <row r="2" spans="1:31" s="5" customFormat="1" ht="59.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="I2" s="3">
-        <v>0.52</v>
-      </c>
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
       <c r="J2" s="3"/>
-      <c r="K2" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="N2" s="3">
-        <v>1200</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="P2" s="3">
-        <v>50</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="R2" s="3">
-        <v>26</v>
-      </c>
-      <c r="S2" s="3">
-        <v>60</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="W2" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="X2" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y2" s="3" t="s">
-        <v>90</v>
-      </c>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
+      <c r="U2" s="3"/>
+      <c r="V2" s="3"/>
+      <c r="W2" s="3"/>
+      <c r="X2" s="3"/>
+      <c r="Y2" s="3"/>
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
-      <c r="AC2" s="3" t="s">
-        <v>54</v>
-      </c>
+      <c r="AC2" s="3"/>
       <c r="AD2" s="4"/>
       <c r="AE2" s="4"/>
     </row>
     <row r="3" spans="1:31" s="5" customFormat="1" ht="59.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>97</v>
-      </c>
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
       <c r="J3" s="3"/>
-      <c r="K3" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="N3" s="3">
-        <v>1200</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q3" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="R3" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="S3" s="3">
-        <v>60</v>
-      </c>
-      <c r="T3" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="U3" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="V3" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="W3" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="X3" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="Y3" s="3" t="s">
-        <v>106</v>
-      </c>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
       <c r="AB3" s="3"/>
-      <c r="AC3" s="3" t="s">
-        <v>54</v>
-      </c>
+      <c r="AC3" s="3"/>
       <c r="AD3" s="4"/>
       <c r="AE3" s="4"/>
     </row>
     <row r="4" spans="1:31" s="5" customFormat="1" ht="59.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>39</v>
-      </c>
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
       <c r="J4" s="3"/>
-      <c r="K4" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="N4" s="3">
-        <v>1200</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="P4" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q4" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="R4" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S4" s="3">
-        <v>60</v>
-      </c>
-      <c r="T4" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="U4" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="V4" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="W4" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="X4" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y4" s="3" t="s">
-        <v>53</v>
-      </c>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
       <c r="Z4" s="3"/>
       <c r="AA4" s="3"/>
       <c r="AB4" s="3"/>
-      <c r="AC4" s="3" t="s">
-        <v>54</v>
-      </c>
+      <c r="AC4" s="3"/>
       <c r="AD4" s="4"/>
       <c r="AE4" s="4"/>
     </row>
     <row r="5" spans="1:31" s="5" customFormat="1" ht="59.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>62</v>
-      </c>
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
       <c r="J5" s="3"/>
-      <c r="K5" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="N5" s="3">
-        <v>1200</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q5" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="R5" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="S5" s="3">
-        <v>60</v>
-      </c>
-      <c r="T5" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="U5" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="V5" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="W5" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="X5" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="Y5" s="3" t="s">
-        <v>73</v>
-      </c>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="Y5" s="3"/>
       <c r="Z5" s="3"/>
       <c r="AA5" s="3"/>
       <c r="AB5" s="3"/>
-      <c r="AC5" s="3" t="s">
-        <v>54</v>
-      </c>
+      <c r="AC5" s="3"/>
       <c r="AD5" s="4"/>
       <c r="AE5" s="4"/>
     </row>

</xml_diff>